<commit_message>
updated component creation loginc
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sajikumarjs/personal/reli_engine/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED654546-E182-0D4E-8467-AB2BD585AB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AACB1A6-F856-9643-B3C0-341207395588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" activeTab="1" xr2:uid="{C431CB80-CA07-A34D-829D-C72251BD8198}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19840" activeTab="1" xr2:uid="{C431CB80-CA07-A34D-829D-C72251BD8198}"/>
   </bookViews>
   <sheets>
     <sheet name="component" sheetId="1" r:id="rId1"/>

</xml_diff>